<commit_message>
ingesta: snapshot 2026-10-18 18:38 UTC
</commit_message>
<xml_diff>
--- a/data_lake/datos_diarios_preliminares/dt=2026-10-18/Temp-max-octubre-26.xlsx
+++ b/data_lake/datos_diarios_preliminares/dt=2026-10-18/Temp-max-octubre-26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.187.8\Oficina\Mi unidad\OSPA\02. Datos Diarios\Tablas\Datos hidrometeorologicos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20265B72-DFA2-4B56-B5DD-84EF4A087D15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F9F226A-6BE1-4549-89E2-DAD0C5B8462C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="355" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9474,7 +9474,9 @@
       <c r="T5" s="63">
         <v>32.299999999999997</v>
       </c>
-      <c r="U5" s="63"/>
+      <c r="U5" s="63">
+        <v>30</v>
+      </c>
       <c r="V5" s="63"/>
       <c r="W5" s="63"/>
       <c r="X5" s="63"/>
@@ -9491,7 +9493,7 @@
       <c r="AI5" s="63"/>
       <c r="AJ5" s="36">
         <f>+IF(SUM($E5:$AI5)&gt;0,LOOKUP(1000,$E5:$AI5),NA())</f>
-        <v>32.299999999999997</v>
+        <v>30</v>
       </c>
       <c r="AK5" s="21">
         <f>+MAX($E5:$AI5)</f>
@@ -9509,11 +9511,11 @@
       </c>
       <c r="AO5" s="23">
         <f>IF(COUNTIF(E5:AI5,"&gt;0")&gt;=15,AVERAGE(E5:AI5),"")</f>
-        <v>32.143749999999997</v>
+        <v>32.017647058823528</v>
       </c>
       <c r="AP5" s="23">
         <f>IF(AN5&gt;0,IFERROR(AO5-AN5,""),"")</f>
-        <v>1.7003905692935177</v>
+        <v>1.5742876281170481</v>
       </c>
       <c r="AQ5" s="20"/>
     </row>
@@ -9578,7 +9580,9 @@
       <c r="T6" s="63">
         <v>32.700000000000003</v>
       </c>
-      <c r="U6" s="63"/>
+      <c r="U6" s="63">
+        <v>30.9</v>
+      </c>
       <c r="V6" s="63"/>
       <c r="W6" s="63"/>
       <c r="X6" s="63"/>
@@ -9595,7 +9599,7 @@
       <c r="AI6" s="63"/>
       <c r="AJ6" s="36">
         <f t="shared" ref="AJ6:AJ48" si="0">+IF(SUM($E6:$AI6)&gt;0,LOOKUP(1000,$E6:$AI6),NA())</f>
-        <v>32.700000000000003</v>
+        <v>30.9</v>
       </c>
       <c r="AK6" s="21">
         <f t="shared" ref="AK6:AK48" si="1">+MAX($E6:$AI6)</f>
@@ -9613,11 +9617,11 @@
       </c>
       <c r="AO6" s="23">
         <f t="shared" ref="AO6:AO15" si="3">IF(COUNTIF(E6:AI6,"&gt;0")&gt;=15,AVERAGE(E6:AI6),"")</f>
-        <v>31.762500000000003</v>
+        <v>31.711764705882356</v>
       </c>
       <c r="AP6" s="23">
         <f t="shared" ref="AP6:AP48" si="4">IF(AN6&gt;0,IFERROR(AO6-AN6,""),"")</f>
-        <v>1.0446514566675837</v>
+        <v>0.99391616254993664</v>
       </c>
       <c r="AQ6" s="20"/>
     </row>
@@ -9682,7 +9686,9 @@
       <c r="T7" s="63">
         <v>34.6</v>
       </c>
-      <c r="U7" s="63"/>
+      <c r="U7" s="63">
+        <v>34.700000000000003</v>
+      </c>
       <c r="V7" s="63"/>
       <c r="W7" s="63"/>
       <c r="X7" s="63"/>
@@ -9699,7 +9705,7 @@
       <c r="AI7" s="63"/>
       <c r="AJ7" s="36">
         <f t="shared" si="0"/>
-        <v>34.6</v>
+        <v>34.700000000000003</v>
       </c>
       <c r="AK7" s="21">
         <f t="shared" si="1"/>
@@ -9717,11 +9723,11 @@
       </c>
       <c r="AO7" s="23">
         <f t="shared" si="3"/>
-        <v>33.981250000000003</v>
+        <v>34.023529411764713</v>
       </c>
       <c r="AP7" s="23">
         <f t="shared" si="4"/>
-        <v>1.5396386133244562</v>
+        <v>1.5819180250891662</v>
       </c>
       <c r="AQ7" s="20"/>
     </row>
@@ -9786,7 +9792,9 @@
       <c r="T8" s="63">
         <v>34.700000000000003</v>
       </c>
-      <c r="U8" s="63"/>
+      <c r="U8" s="63">
+        <v>33.1</v>
+      </c>
       <c r="V8" s="63"/>
       <c r="W8" s="63"/>
       <c r="X8" s="63"/>
@@ -9803,7 +9811,7 @@
       <c r="AI8" s="63"/>
       <c r="AJ8" s="36">
         <f t="shared" si="0"/>
-        <v>34.700000000000003</v>
+        <v>33.1</v>
       </c>
       <c r="AK8" s="21">
         <f t="shared" si="1"/>
@@ -9821,11 +9829,11 @@
       </c>
       <c r="AO8" s="23">
         <f t="shared" si="3"/>
-        <v>32.800000000000004</v>
+        <v>32.817647058823532</v>
       </c>
       <c r="AP8" s="23">
         <f t="shared" si="4"/>
-        <v>1.1304226918798754</v>
+        <v>1.148069750703403</v>
       </c>
       <c r="AQ8" s="20"/>
     </row>
@@ -9890,7 +9898,9 @@
       <c r="T9" s="63">
         <v>36.9</v>
       </c>
-      <c r="U9" s="63"/>
+      <c r="U9" s="63">
+        <v>35.9</v>
+      </c>
       <c r="V9" s="63"/>
       <c r="W9" s="63"/>
       <c r="X9" s="63"/>
@@ -9907,7 +9917,7 @@
       <c r="AI9" s="63"/>
       <c r="AJ9" s="36">
         <f t="shared" si="0"/>
-        <v>36.9</v>
+        <v>35.9</v>
       </c>
       <c r="AK9" s="21">
         <f t="shared" si="1"/>
@@ -9925,11 +9935,11 @@
       </c>
       <c r="AO9" s="23">
         <f t="shared" si="3"/>
-        <v>34.35</v>
+        <v>34.441176470588232</v>
       </c>
       <c r="AP9" s="23">
         <f t="shared" si="4"/>
-        <v>1.5882361425648739</v>
+        <v>1.6794126131531044</v>
       </c>
       <c r="AQ9" s="20"/>
     </row>
@@ -9994,7 +10004,9 @@
       <c r="T10" s="63">
         <v>35.5</v>
       </c>
-      <c r="U10" s="63"/>
+      <c r="U10" s="63">
+        <v>34.9</v>
+      </c>
       <c r="V10" s="63"/>
       <c r="W10" s="63"/>
       <c r="X10" s="63"/>
@@ -10011,7 +10023,7 @@
       <c r="AI10" s="63"/>
       <c r="AJ10" s="36">
         <f t="shared" si="0"/>
-        <v>35.5</v>
+        <v>34.9</v>
       </c>
       <c r="AK10" s="21">
         <f t="shared" si="1"/>
@@ -10029,11 +10041,11 @@
       </c>
       <c r="AO10" s="23">
         <f t="shared" si="3"/>
-        <v>34.199999999999996</v>
+        <v>34.241176470588229</v>
       </c>
       <c r="AP10" s="23">
         <f t="shared" si="4"/>
-        <v>1.4140356442910829</v>
+        <v>1.4552121148793162</v>
       </c>
       <c r="AQ10" s="20"/>
     </row>
@@ -10098,7 +10110,9 @@
       <c r="T11" s="63">
         <v>36.700000000000003</v>
       </c>
-      <c r="U11" s="63"/>
+      <c r="U11" s="63">
+        <v>34.4</v>
+      </c>
       <c r="V11" s="63"/>
       <c r="W11" s="63"/>
       <c r="X11" s="63"/>
@@ -10115,7 +10129,7 @@
       <c r="AI11" s="63"/>
       <c r="AJ11" s="36">
         <f t="shared" si="0"/>
-        <v>36.700000000000003</v>
+        <v>34.4</v>
       </c>
       <c r="AK11" s="21">
         <f t="shared" si="1"/>
@@ -10133,11 +10147,11 @@
       </c>
       <c r="AO11" s="23">
         <f t="shared" si="3"/>
-        <v>34.818750000000009</v>
+        <v>34.794117647058833</v>
       </c>
       <c r="AP11" s="23">
         <f t="shared" si="4"/>
-        <v>1.781302767821586</v>
+        <v>1.7566704148804106</v>
       </c>
       <c r="AQ11" s="20"/>
     </row>
@@ -10202,7 +10216,9 @@
       <c r="T12" s="63">
         <v>35</v>
       </c>
-      <c r="U12" s="63"/>
+      <c r="U12" s="63">
+        <v>29.4</v>
+      </c>
       <c r="V12" s="63"/>
       <c r="W12" s="63"/>
       <c r="X12" s="63"/>
@@ -10219,7 +10235,7 @@
       <c r="AI12" s="63"/>
       <c r="AJ12" s="36">
         <f t="shared" si="0"/>
-        <v>35</v>
+        <v>29.4</v>
       </c>
       <c r="AK12" s="21">
         <f t="shared" si="1"/>
@@ -10237,11 +10253,11 @@
       </c>
       <c r="AO12" s="23">
         <f t="shared" si="3"/>
-        <v>31.824999999999999</v>
+        <v>31.682352941176472</v>
       </c>
       <c r="AP12" s="23">
         <f t="shared" si="4"/>
-        <v>0.71270609318996847</v>
+        <v>0.5700590343664409</v>
       </c>
       <c r="AQ12" s="20"/>
     </row>
@@ -10306,7 +10322,9 @@
       <c r="T13" s="63">
         <v>35.4</v>
       </c>
-      <c r="U13" s="63"/>
+      <c r="U13" s="63">
+        <v>32.200000000000003</v>
+      </c>
       <c r="V13" s="63"/>
       <c r="W13" s="63"/>
       <c r="X13" s="63"/>
@@ -10323,7 +10341,7 @@
       <c r="AI13" s="63"/>
       <c r="AJ13" s="36">
         <f t="shared" si="0"/>
-        <v>35.4</v>
+        <v>32.200000000000003</v>
       </c>
       <c r="AK13" s="21">
         <f t="shared" si="1"/>
@@ -10341,11 +10359,11 @@
       </c>
       <c r="AO13" s="23">
         <f t="shared" si="3"/>
-        <v>32.5625</v>
+        <v>32.54117647058824</v>
       </c>
       <c r="AP13" s="23">
         <f t="shared" si="4"/>
-        <v>0.87816666666666876</v>
+        <v>0.85684313725490924</v>
       </c>
       <c r="AQ13" s="20"/>
     </row>
@@ -10410,7 +10428,9 @@
       <c r="T14" s="63">
         <v>35.1</v>
       </c>
-      <c r="U14" s="63"/>
+      <c r="U14" s="63">
+        <v>29.7</v>
+      </c>
       <c r="V14" s="63"/>
       <c r="W14" s="63"/>
       <c r="X14" s="63"/>
@@ -10427,7 +10447,7 @@
       <c r="AI14" s="63"/>
       <c r="AJ14" s="36">
         <f t="shared" si="0"/>
-        <v>35.1</v>
+        <v>29.7</v>
       </c>
       <c r="AK14" s="21">
         <f t="shared" si="1"/>
@@ -10445,11 +10465,11 @@
       </c>
       <c r="AO14" s="23">
         <f t="shared" si="3"/>
-        <v>33.043750000000003</v>
+        <v>32.847058823529416</v>
       </c>
       <c r="AP14" s="23">
         <f t="shared" si="4"/>
-        <v>0.60052416892667537</v>
+        <v>0.40383299245608839</v>
       </c>
       <c r="AQ14" s="20"/>
     </row>
@@ -10514,7 +10534,9 @@
       <c r="T15" s="63">
         <v>31.7</v>
       </c>
-      <c r="U15" s="63"/>
+      <c r="U15" s="63">
+        <v>32</v>
+      </c>
       <c r="V15" s="63"/>
       <c r="W15" s="63"/>
       <c r="X15" s="63"/>
@@ -10531,7 +10553,7 @@
       <c r="AI15" s="63"/>
       <c r="AJ15" s="36">
         <f t="shared" si="0"/>
-        <v>31.7</v>
+        <v>32</v>
       </c>
       <c r="AK15" s="21">
         <f t="shared" si="1"/>
@@ -10549,11 +10571,11 @@
       </c>
       <c r="AO15" s="23">
         <f t="shared" si="3"/>
-        <v>31.700000000000003</v>
+        <v>31.71764705882353</v>
       </c>
       <c r="AP15" s="23">
         <f t="shared" si="4"/>
-        <v>-4.4999041080128421E-2</v>
+        <v>-2.7351982256600849E-2</v>
       </c>
       <c r="AQ15" s="20"/>
     </row>
@@ -10667,7 +10689,9 @@
       <c r="T17" s="63">
         <v>32</v>
       </c>
-      <c r="U17" s="63"/>
+      <c r="U17" s="63">
+        <v>30.5</v>
+      </c>
       <c r="V17" s="63"/>
       <c r="W17" s="63"/>
       <c r="X17" s="63"/>
@@ -10684,7 +10708,7 @@
       <c r="AI17" s="63"/>
       <c r="AJ17" s="36">
         <f t="shared" si="0"/>
-        <v>32</v>
+        <v>30.5</v>
       </c>
       <c r="AK17" s="21">
         <f t="shared" si="1"/>
@@ -10702,11 +10726,11 @@
       </c>
       <c r="AO17" s="23">
         <f>IF(COUNTIF(E17:AI17,"&gt;0")&gt;=15,AVERAGE(E17:AI17),"")</f>
-        <v>32.274999999999999</v>
+        <v>32.170588235294119</v>
       </c>
       <c r="AP17" s="23">
         <f>IF(AN17&gt;0,IFERROR(AO17-AN17,""),"")</f>
-        <v>0.84066984858458937</v>
+        <v>0.73625808387870961</v>
       </c>
       <c r="AQ17" s="20"/>
     </row>
@@ -10771,7 +10795,9 @@
       <c r="T18" s="63">
         <v>27.8</v>
       </c>
-      <c r="U18" s="63"/>
+      <c r="U18" s="63">
+        <v>27.8</v>
+      </c>
       <c r="V18" s="63"/>
       <c r="W18" s="63"/>
       <c r="X18" s="63"/>
@@ -10806,11 +10832,11 @@
       </c>
       <c r="AO18" s="23">
         <f t="shared" ref="AO18:AO33" si="5">IF(COUNTIF(E18:AI18,"&gt;0")&gt;=15,AVERAGE(E18:AI18),"")</f>
-        <v>27.612500000000001</v>
+        <v>27.623529411764707</v>
       </c>
       <c r="AP18" s="23">
         <f t="shared" si="4"/>
-        <v>1.9639929693961911</v>
+        <v>1.9750223811608976</v>
       </c>
       <c r="AQ18" s="20"/>
     </row>
@@ -10875,7 +10901,9 @@
       <c r="T19" s="63">
         <v>37</v>
       </c>
-      <c r="U19" s="63"/>
+      <c r="U19" s="63">
+        <v>37</v>
+      </c>
       <c r="V19" s="63"/>
       <c r="W19" s="63"/>
       <c r="X19" s="63"/>
@@ -10910,11 +10938,11 @@
       </c>
       <c r="AO19" s="23">
         <f t="shared" si="5"/>
-        <v>34.931249999999991</v>
+        <v>35.052941176470583</v>
       </c>
       <c r="AP19" s="23">
         <f t="shared" si="4"/>
-        <v>1.916234146677688</v>
+        <v>2.0379253231482792</v>
       </c>
       <c r="AQ19" s="20"/>
     </row>
@@ -10979,7 +11007,9 @@
       <c r="T20" s="63">
         <v>25.5</v>
       </c>
-      <c r="U20" s="63"/>
+      <c r="U20" s="63">
+        <v>30</v>
+      </c>
       <c r="V20" s="63"/>
       <c r="W20" s="63"/>
       <c r="X20" s="63"/>
@@ -10996,7 +11026,7 @@
       <c r="AI20" s="63"/>
       <c r="AJ20" s="36">
         <f t="shared" si="0"/>
-        <v>25.5</v>
+        <v>30</v>
       </c>
       <c r="AK20" s="21">
         <f t="shared" si="1"/>
@@ -11014,11 +11044,11 @@
       </c>
       <c r="AO20" s="23">
         <f t="shared" si="5"/>
-        <v>28.368749999999999</v>
+        <v>28.464705882352941</v>
       </c>
       <c r="AP20" s="23">
         <f t="shared" si="4"/>
-        <v>1.0765144381368792</v>
+        <v>1.1724703204898219</v>
       </c>
       <c r="AQ20" s="20"/>
     </row>
@@ -11083,7 +11113,9 @@
       <c r="T21" s="63">
         <v>21.7</v>
       </c>
-      <c r="U21" s="63"/>
+      <c r="U21" s="63">
+        <v>23.8</v>
+      </c>
       <c r="V21" s="63"/>
       <c r="W21" s="63"/>
       <c r="X21" s="63"/>
@@ -11100,7 +11132,7 @@
       <c r="AI21" s="63"/>
       <c r="AJ21" s="36">
         <f t="shared" si="0"/>
-        <v>21.7</v>
+        <v>23.8</v>
       </c>
       <c r="AK21" s="21">
         <f t="shared" si="1"/>
@@ -11118,11 +11150,11 @@
       </c>
       <c r="AO21" s="23">
         <f t="shared" si="5"/>
-        <v>23.35</v>
+        <v>23.376470588235296</v>
       </c>
       <c r="AP21" s="23">
         <f t="shared" si="4"/>
-        <v>1.4067741935483902</v>
+        <v>1.4332447817836851</v>
       </c>
       <c r="AQ21" s="20"/>
     </row>
@@ -11253,7 +11285,9 @@
       <c r="T23" s="63">
         <v>24.7</v>
       </c>
-      <c r="U23" s="63"/>
+      <c r="U23" s="63">
+        <v>27.6</v>
+      </c>
       <c r="V23" s="63"/>
       <c r="W23" s="63"/>
       <c r="X23" s="63"/>
@@ -11270,7 +11304,7 @@
       <c r="AI23" s="63"/>
       <c r="AJ23" s="36">
         <f t="shared" si="0"/>
-        <v>24.7</v>
+        <v>27.6</v>
       </c>
       <c r="AK23" s="21">
         <f t="shared" si="1"/>
@@ -11288,11 +11322,11 @@
       </c>
       <c r="AO23" s="23">
         <f t="shared" si="5"/>
-        <v>27.681249999999995</v>
+        <v>27.67647058823529</v>
       </c>
       <c r="AP23" s="23">
         <f t="shared" si="4"/>
-        <v>1.4937810173697237</v>
+        <v>1.4890016056050186</v>
       </c>
       <c r="AQ23" s="20"/>
     </row>
@@ -11357,7 +11391,9 @@
       <c r="T24" s="63">
         <v>28.1</v>
       </c>
-      <c r="U24" s="63"/>
+      <c r="U24" s="63">
+        <v>28.1</v>
+      </c>
       <c r="V24" s="63"/>
       <c r="W24" s="63"/>
       <c r="X24" s="63"/>
@@ -11392,11 +11428,11 @@
       </c>
       <c r="AO24" s="23">
         <f t="shared" si="5"/>
-        <v>28.262499999999999</v>
+        <v>28.252941176470589</v>
       </c>
       <c r="AP24" s="23">
         <f t="shared" si="4"/>
-        <v>0.89993919610854789</v>
+        <v>0.89038037257913771</v>
       </c>
       <c r="AQ24" s="20"/>
     </row>
@@ -11461,7 +11497,9 @@
       <c r="T25" s="63">
         <v>30.3</v>
       </c>
-      <c r="U25" s="63"/>
+      <c r="U25" s="63">
+        <v>32</v>
+      </c>
       <c r="V25" s="63"/>
       <c r="W25" s="63"/>
       <c r="X25" s="63"/>
@@ -11478,7 +11516,7 @@
       <c r="AI25" s="63"/>
       <c r="AJ25" s="36">
         <f t="shared" si="0"/>
-        <v>30.3</v>
+        <v>32</v>
       </c>
       <c r="AK25" s="21">
         <f t="shared" si="1"/>
@@ -11496,11 +11534,11 @@
       </c>
       <c r="AO25" s="23">
         <f t="shared" si="5"/>
-        <v>29.731249999999999</v>
+        <v>29.86470588235294</v>
       </c>
       <c r="AP25" s="23">
         <f t="shared" si="4"/>
-        <v>0.8673471311755705</v>
+        <v>1.0008030135285111</v>
       </c>
       <c r="AQ25" s="20"/>
     </row>
@@ -11565,7 +11603,9 @@
       <c r="T26" s="63">
         <v>21.6</v>
       </c>
-      <c r="U26" s="63"/>
+      <c r="U26" s="63">
+        <v>21.8</v>
+      </c>
       <c r="V26" s="63"/>
       <c r="W26" s="63"/>
       <c r="X26" s="63"/>
@@ -11582,7 +11622,7 @@
       <c r="AI26" s="63"/>
       <c r="AJ26" s="36">
         <f t="shared" si="0"/>
-        <v>21.6</v>
+        <v>21.8</v>
       </c>
       <c r="AK26" s="21">
         <f t="shared" si="1"/>
@@ -11600,11 +11640,11 @@
       </c>
       <c r="AO26" s="23">
         <f t="shared" si="5"/>
-        <v>21.143750000000001</v>
+        <v>21.182352941176472</v>
       </c>
       <c r="AP26" s="23">
         <f t="shared" si="4"/>
-        <v>1.7231158308897498</v>
+        <v>1.7617187720662209</v>
       </c>
       <c r="AQ26" s="20"/>
     </row>
@@ -11669,7 +11709,9 @@
       <c r="T27" s="63">
         <v>22.2</v>
       </c>
-      <c r="U27" s="63"/>
+      <c r="U27" s="63">
+        <v>23</v>
+      </c>
       <c r="V27" s="63"/>
       <c r="W27" s="63"/>
       <c r="X27" s="63"/>
@@ -11686,7 +11728,7 @@
       <c r="AI27" s="63"/>
       <c r="AJ27" s="36">
         <f t="shared" si="0"/>
-        <v>22.2</v>
+        <v>23</v>
       </c>
       <c r="AK27" s="21">
         <f t="shared" si="1"/>
@@ -11704,11 +11746,11 @@
       </c>
       <c r="AO27" s="23">
         <f t="shared" si="5"/>
-        <v>22.1875</v>
+        <v>22.235294117647058</v>
       </c>
       <c r="AP27" s="23">
         <f t="shared" si="4"/>
-        <v>3.5328316575897212</v>
+        <v>3.5806257752367792</v>
       </c>
       <c r="AQ27" s="20"/>
     </row>
@@ -11773,7 +11815,9 @@
       <c r="T28" s="63">
         <v>29.9</v>
       </c>
-      <c r="U28" s="63"/>
+      <c r="U28" s="63">
+        <v>30.8</v>
+      </c>
       <c r="V28" s="63"/>
       <c r="W28" s="63"/>
       <c r="X28" s="63"/>
@@ -11790,7 +11834,7 @@
       <c r="AI28" s="63"/>
       <c r="AJ28" s="36">
         <f t="shared" si="0"/>
-        <v>29.9</v>
+        <v>30.8</v>
       </c>
       <c r="AK28" s="21">
         <f t="shared" si="1"/>
@@ -11808,11 +11852,11 @@
       </c>
       <c r="AO28" s="23">
         <f t="shared" si="5"/>
-        <v>30.750000000000004</v>
+        <v>30.752941176470593</v>
       </c>
       <c r="AP28" s="23">
         <f t="shared" si="4"/>
-        <v>1.1293432202206439</v>
+        <v>1.132284396691233</v>
       </c>
       <c r="AQ28" s="20"/>
     </row>
@@ -11941,7 +11985,9 @@
       <c r="T30" s="63">
         <v>36.4</v>
       </c>
-      <c r="U30" s="63"/>
+      <c r="U30" s="63">
+        <v>35.700000000000003</v>
+      </c>
       <c r="V30" s="63"/>
       <c r="W30" s="63"/>
       <c r="X30" s="63"/>
@@ -11958,7 +12004,7 @@
       <c r="AI30" s="63"/>
       <c r="AJ30" s="36">
         <f t="shared" si="0"/>
-        <v>36.4</v>
+        <v>35.700000000000003</v>
       </c>
       <c r="AK30" s="21">
         <f t="shared" si="1"/>
@@ -11976,11 +12022,11 @@
       </c>
       <c r="AO30" s="23">
         <f t="shared" si="5"/>
-        <v>35.674999999999997</v>
+        <v>35.676470588235297</v>
       </c>
       <c r="AP30" s="23">
         <f t="shared" si="4"/>
-        <v>2.2767204301075239</v>
+        <v>2.2781910183428238</v>
       </c>
       <c r="AQ30" s="20"/>
     </row>
@@ -12045,7 +12091,9 @@
       <c r="T31" s="63">
         <v>23.4</v>
       </c>
-      <c r="U31" s="63"/>
+      <c r="U31" s="63">
+        <v>26.2</v>
+      </c>
       <c r="V31" s="63"/>
       <c r="W31" s="63"/>
       <c r="X31" s="63"/>
@@ -12062,7 +12110,7 @@
       <c r="AI31" s="63"/>
       <c r="AJ31" s="36">
         <f t="shared" si="0"/>
-        <v>23.4</v>
+        <v>26.2</v>
       </c>
       <c r="AK31" s="21">
         <f t="shared" si="1"/>
@@ -12080,11 +12128,11 @@
       </c>
       <c r="AO31" s="23">
         <f t="shared" si="5"/>
-        <v>25.681249999999999</v>
+        <v>25.711764705882352</v>
       </c>
       <c r="AP31" s="23">
         <f t="shared" si="4"/>
-        <v>1.3612569212705488</v>
+        <v>1.3917716271529024</v>
       </c>
       <c r="AQ31" s="20"/>
     </row>
@@ -12149,7 +12197,9 @@
       <c r="T32" s="63">
         <v>17.2</v>
       </c>
-      <c r="U32" s="63"/>
+      <c r="U32" s="63">
+        <v>18.8</v>
+      </c>
       <c r="V32" s="63"/>
       <c r="W32" s="63"/>
       <c r="X32" s="63"/>
@@ -12166,7 +12216,7 @@
       <c r="AI32" s="63"/>
       <c r="AJ32" s="36">
         <f t="shared" si="0"/>
-        <v>17.2</v>
+        <v>18.8</v>
       </c>
       <c r="AK32" s="21">
         <f t="shared" si="1"/>
@@ -12184,11 +12234,11 @@
       </c>
       <c r="AO32" s="23">
         <f t="shared" si="5"/>
-        <v>19.787500000000001</v>
+        <v>19.729411764705883</v>
       </c>
       <c r="AP32" s="23">
         <f t="shared" si="4"/>
-        <v>1.8668258846373398</v>
+        <v>1.8087376493432217</v>
       </c>
       <c r="AQ32" s="20"/>
     </row>
@@ -12253,7 +12303,9 @@
       <c r="T33" s="63">
         <v>16.600000000000001</v>
       </c>
-      <c r="U33" s="63"/>
+      <c r="U33" s="63">
+        <v>16.399999999999999</v>
+      </c>
       <c r="V33" s="63"/>
       <c r="W33" s="63"/>
       <c r="X33" s="63"/>
@@ -12270,7 +12322,7 @@
       <c r="AI33" s="63"/>
       <c r="AJ33" s="36">
         <f t="shared" si="0"/>
-        <v>16.600000000000001</v>
+        <v>16.399999999999999</v>
       </c>
       <c r="AK33" s="21">
         <f t="shared" si="1"/>
@@ -12288,11 +12340,11 @@
       </c>
       <c r="AO33" s="23">
         <f t="shared" si="5"/>
-        <v>18.125000000000004</v>
+        <v>18.023529411764709</v>
       </c>
       <c r="AP33" s="23">
         <f t="shared" si="4"/>
-        <v>1.2294225384526847</v>
+        <v>1.1279519502173905</v>
       </c>
       <c r="AQ33" s="20"/>
       <c r="AT33" s="15"/>
@@ -12409,7 +12461,9 @@
       <c r="T35" s="63">
         <v>25.8</v>
       </c>
-      <c r="U35" s="63"/>
+      <c r="U35" s="63">
+        <v>32.799999999999997</v>
+      </c>
       <c r="V35" s="63"/>
       <c r="W35" s="63"/>
       <c r="X35" s="63"/>
@@ -12426,7 +12480,7 @@
       <c r="AI35" s="63"/>
       <c r="AJ35" s="36">
         <f t="shared" si="0"/>
-        <v>25.8</v>
+        <v>32.799999999999997</v>
       </c>
       <c r="AK35" s="21">
         <f t="shared" si="1"/>
@@ -12444,11 +12498,11 @@
       </c>
       <c r="AO35" s="23">
         <f>IF(COUNTIF(E35:AI35,"&gt;0")&gt;=15,AVERAGE(E35:AI35),"")</f>
-        <v>31.275000000000002</v>
+        <v>31.364705882352943</v>
       </c>
       <c r="AP35" s="23">
         <f t="shared" si="4"/>
-        <v>0.72063180034010088</v>
+        <v>0.81033768269304218</v>
       </c>
       <c r="AQ35" s="20"/>
       <c r="AT35" s="15"/>
@@ -12632,7 +12686,9 @@
       <c r="T38" s="63">
         <v>33.1</v>
       </c>
-      <c r="U38" s="63"/>
+      <c r="U38" s="63">
+        <v>34.6</v>
+      </c>
       <c r="V38" s="63"/>
       <c r="W38" s="63"/>
       <c r="X38" s="63"/>
@@ -12649,7 +12705,7 @@
       <c r="AI38" s="63"/>
       <c r="AJ38" s="36">
         <f t="shared" si="0"/>
-        <v>33.1</v>
+        <v>34.6</v>
       </c>
       <c r="AK38" s="21">
         <f t="shared" si="1"/>
@@ -12667,11 +12723,11 @@
       </c>
       <c r="AO38" s="23">
         <f>IF(COUNTIF(E38:AI38,"&gt;0")&gt;=15,AVERAGE(E38:AI38),"")</f>
-        <v>33.274999999999991</v>
+        <v>33.35294117647058</v>
       </c>
       <c r="AP38" s="23">
         <f t="shared" si="4"/>
-        <v>1.3380135335558023</v>
+        <v>1.4159547100263907</v>
       </c>
       <c r="AQ38" s="20"/>
       <c r="AT38" s="15"/>
@@ -12737,7 +12793,9 @@
       <c r="T39" s="63">
         <v>35.9</v>
       </c>
-      <c r="U39" s="63"/>
+      <c r="U39" s="63">
+        <v>33.4</v>
+      </c>
       <c r="V39" s="63"/>
       <c r="W39" s="63"/>
       <c r="X39" s="63"/>
@@ -12754,7 +12812,7 @@
       <c r="AI39" s="63"/>
       <c r="AJ39" s="36">
         <f t="shared" si="0"/>
-        <v>35.9</v>
+        <v>33.4</v>
       </c>
       <c r="AK39" s="21">
         <f t="shared" si="1"/>
@@ -12772,11 +12830,11 @@
       </c>
       <c r="AO39" s="23">
         <f t="shared" ref="AO39:AO48" si="7">IF(COUNTIF(E39:AI39,"&gt;0")&gt;=15,AVERAGE(E39:AI39),"")</f>
-        <v>34.493749999999999</v>
+        <v>34.429411764705883</v>
       </c>
       <c r="AP39" s="23">
         <f t="shared" si="4"/>
-        <v>1.0710224014337015</v>
+        <v>1.0066841661395856</v>
       </c>
       <c r="AQ39" s="20"/>
       <c r="AT39" s="15"/>
@@ -12842,7 +12900,9 @@
       <c r="T40" s="63">
         <v>32.299999999999997</v>
       </c>
-      <c r="U40" s="63"/>
+      <c r="U40" s="63">
+        <v>31.2</v>
+      </c>
       <c r="V40" s="63"/>
       <c r="W40" s="63"/>
       <c r="X40" s="63"/>
@@ -12859,7 +12919,7 @@
       <c r="AI40" s="63"/>
       <c r="AJ40" s="36">
         <f t="shared" si="0"/>
-        <v>32.299999999999997</v>
+        <v>31.2</v>
       </c>
       <c r="AK40" s="21">
         <f t="shared" si="1"/>
@@ -12877,11 +12937,11 @@
       </c>
       <c r="AO40" s="23">
         <f t="shared" si="7"/>
-        <v>31.137499999999999</v>
+        <v>31.141176470588235</v>
       </c>
       <c r="AP40" s="23">
         <f t="shared" si="4"/>
-        <v>0.25912365591397801</v>
+        <v>0.26280012650221352</v>
       </c>
       <c r="AQ40" s="20"/>
       <c r="AT40" s="15"/>
@@ -12943,7 +13003,9 @@
       <c r="T41" s="63">
         <v>33.4</v>
       </c>
-      <c r="U41" s="63"/>
+      <c r="U41" s="63">
+        <v>29.4</v>
+      </c>
       <c r="V41" s="63"/>
       <c r="W41" s="63"/>
       <c r="X41" s="63"/>
@@ -12960,7 +13022,7 @@
       <c r="AI41" s="63"/>
       <c r="AJ41" s="36">
         <f t="shared" si="0"/>
-        <v>33.4</v>
+        <v>29.4</v>
       </c>
       <c r="AK41" s="21">
         <f t="shared" si="1"/>
@@ -12976,13 +13038,13 @@
       <c r="AN41" s="23">
         <v>31.008190582128289</v>
       </c>
-      <c r="AO41" s="23" t="str">
+      <c r="AO41" s="23">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="AP41" s="23" t="str">
+        <v>32.199999999999996</v>
+      </c>
+      <c r="AP41" s="23">
         <f t="shared" si="4"/>
-        <v/>
+        <v>1.1918094178717062</v>
       </c>
       <c r="AQ41" s="20"/>
       <c r="AT41" s="15"/>
@@ -13114,7 +13176,9 @@
       <c r="T43" s="63">
         <v>33</v>
       </c>
-      <c r="U43" s="63"/>
+      <c r="U43" s="63">
+        <v>33.200000000000003</v>
+      </c>
       <c r="V43" s="63"/>
       <c r="W43" s="63"/>
       <c r="X43" s="63"/>
@@ -13131,7 +13195,7 @@
       <c r="AI43" s="63"/>
       <c r="AJ43" s="36">
         <f t="shared" si="0"/>
-        <v>33</v>
+        <v>33.200000000000003</v>
       </c>
       <c r="AK43" s="21">
         <f t="shared" si="1"/>
@@ -13149,11 +13213,11 @@
       </c>
       <c r="AO43" s="23">
         <f t="shared" si="7"/>
-        <v>33.159999999999997</v>
+        <v>33.162499999999994</v>
       </c>
       <c r="AP43" s="23">
         <f t="shared" si="4"/>
-        <v>0.90300732904704972</v>
+        <v>0.90550732904704745</v>
       </c>
       <c r="AQ43" s="20"/>
       <c r="AT43" s="15"/>
@@ -13219,7 +13283,9 @@
       <c r="T44" s="29">
         <v>31.3</v>
       </c>
-      <c r="U44" s="29"/>
+      <c r="U44" s="29">
+        <v>33.1</v>
+      </c>
       <c r="V44" s="29"/>
       <c r="W44" s="29"/>
       <c r="X44" s="29"/>
@@ -13236,7 +13302,7 @@
       <c r="AI44" s="63"/>
       <c r="AJ44" s="36">
         <f t="shared" si="0"/>
-        <v>31.3</v>
+        <v>33.1</v>
       </c>
       <c r="AK44" s="21">
         <f t="shared" si="1"/>
@@ -13254,11 +13320,11 @@
       </c>
       <c r="AO44" s="23">
         <f t="shared" si="7"/>
-        <v>31.881250000000005</v>
+        <v>31.952941176470592</v>
       </c>
       <c r="AP44" s="23">
         <f t="shared" si="4"/>
-        <v>0.79456299915838358</v>
+        <v>0.86625417562897056</v>
       </c>
       <c r="AQ44" s="20"/>
       <c r="AT44" s="15"/>
@@ -13324,7 +13390,9 @@
       <c r="T45" s="63">
         <v>33.799999999999997</v>
       </c>
-      <c r="U45" s="63"/>
+      <c r="U45" s="63">
+        <v>31.4</v>
+      </c>
       <c r="V45" s="63"/>
       <c r="W45" s="63"/>
       <c r="X45" s="63"/>
@@ -13341,7 +13409,7 @@
       <c r="AI45" s="63"/>
       <c r="AJ45" s="36">
         <f t="shared" si="0"/>
-        <v>33.799999999999997</v>
+        <v>31.4</v>
       </c>
       <c r="AK45" s="21">
         <f t="shared" si="1"/>
@@ -13359,11 +13427,11 @@
       </c>
       <c r="AO45" s="23">
         <f t="shared" si="7"/>
-        <v>32.912500000000001</v>
+        <v>32.823529411764703</v>
       </c>
       <c r="AP45" s="23">
         <f t="shared" si="4"/>
-        <v>1.3173052294044112</v>
+        <v>1.2283346411691127</v>
       </c>
       <c r="AQ45" s="20"/>
       <c r="AT45" s="15"/>
@@ -13561,7 +13629,9 @@
       <c r="T48" s="63">
         <v>35.200000000000003</v>
       </c>
-      <c r="U48" s="63"/>
+      <c r="U48" s="63">
+        <v>32.200000000000003</v>
+      </c>
       <c r="V48" s="63"/>
       <c r="W48" s="63"/>
       <c r="X48" s="63"/>
@@ -13578,7 +13648,7 @@
       <c r="AI48" s="63"/>
       <c r="AJ48" s="36">
         <f t="shared" si="0"/>
-        <v>35.200000000000003</v>
+        <v>32.200000000000003</v>
       </c>
       <c r="AK48" s="21">
         <f t="shared" si="1"/>
@@ -13596,11 +13666,11 @@
       </c>
       <c r="AO48" s="23">
         <f t="shared" si="7"/>
-        <v>33.737500000000004</v>
+        <v>33.64705882352942</v>
       </c>
       <c r="AP48" s="23">
         <f t="shared" si="4"/>
-        <v>1.745310752688173</v>
+        <v>1.6548695762175889</v>
       </c>
       <c r="AQ48" s="20"/>
     </row>
@@ -26656,6 +26726,12 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
     <mergeCell ref="M1:M2"/>
     <mergeCell ref="N1:N2"/>
     <mergeCell ref="O1:O2"/>
@@ -26665,12 +26741,6 @@
     <mergeCell ref="J1:J2"/>
     <mergeCell ref="K1:K2"/>
     <mergeCell ref="L1:L2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:E2"/>
   </mergeCells>
   <conditionalFormatting sqref="D4:O13 D15:O31 D33:O34 D36:O46">
     <cfRule type="cellIs" dxfId="0" priority="1" stopIfTrue="1" operator="equal">

</xml_diff>